<commit_message>
feat: lectura de PDF por capas (PyMuPDF, OCR, visión), anclaje de datos y trazas
- extraccion.py: texto nativo por bloques, OCR con Tesseract spa+eng (giro, inclinación,
  4 preprocesados, elección por palabras fiables), OCR por región para sellos y visión
  del modelo si la resolución es menor a 150 dpi
- anclaje.py: número, monto y fecha extraídos deben aparecer en el texto; si no, relectura
  con visión o LECTURA_DUDOSA (POL-GAR-09)
- telemetry.py: spans OpenTelemetry anidados con la traza del workflow en Foundry
- muestras escaneadas (limpia, degradada) y mixta con sello; evaluación por tipo de lectura
- ETL omite los ya procesados antes de extraer; reintentos ante errores transitorios
- imagen Docker y CI con Tesseract en español
</commit_message>
<xml_diff>
--- a/dataplane/samples/registro_tesoreria.xlsx
+++ b/dataplane/samples/registro_tesoreria.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -756,31 +756,130 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>CF-2026-0012</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Agropecuaria Santa Rosa SAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ministerio de Agricultura y Riego</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>130000</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>46497</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>VIGENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CF-2026-0013</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Constructora Los Andes SRL</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Gobierno Regional de Cajamarca</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>78500.25</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>46539</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>VIGENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CF-2026-0014</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Frutas del Valle SA</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Municipalidad Provincial de Chepén</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>54000</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>46455</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>VIGENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>CF-2026-0011</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Agrícola Virú SA</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Gobierno Regional La Libertad</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D14" t="n">
         <v>120000</v>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>PEN</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="n">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="n">
         <v>46446</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>VIGENTE</t>
         </is>

</xml_diff>